<commit_message>
Ajoute le brief du 2e article "Combien ça coûte vraiment" : Dacia Duster vs Peugeot 2008
Sujet identifié par recherche web (rôle Journaliste, skills/agents-ia.md) : Peugeot 2008 (n°1
des SUV vendus en France, jan-août 2026, 33 508 immat./3,1%) vs Dacia Duster (n°4, 19 807
immat./1,8%, source caroom.fr) — même logique éditoriale que Sandero/Clio (petit prix vs
marque généraliste), transposée au segment SUV compact. Aucun article existant du site ne
couvre déjà cette comparaison (vérifié via data/maillage/maillage.json).

Brief sauvegardé dans data/tests/briefs/duster-2008-cout-possession.json, ligne ajoutée dans
tracking-mots-cles.xlsx (statut "en rédaction"), conformément aux étapes 5-6 de
.claude/commands/agent-brief.md. Étape suivante (/agent-test, configuration réelle sur
dacia.fr et peugeot.fr) en attente de confirmation utilisateur.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014Wu7AgBS9aLRsqa1k7Jg2q
</commit_message>
<xml_diff>
--- a/data/keywords/tracking-mots-cles.xlsx
+++ b/data/keywords/tracking-mots-cles.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Légende" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Suivi" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Légende" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suivi" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -839,7 +839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1400"/>
+  <dimension ref="A1:L1402"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64708,6 +64708,90 @@
         </is>
       </c>
     </row>
+    <row r="1401">
+      <c r="A1401" t="inlineStr">
+        <is>
+          <t>dacia sandero vs renault clio</t>
+        </is>
+      </c>
+      <c r="B1401" t="inlineStr">
+        <is>
+          <t>prix réel dacia sandero 2026;prix réel renault clio 2026;citadine la moins chère 2026;coût de possession citadine 2026</t>
+        </is>
+      </c>
+      <c r="C1401" t="inlineStr">
+        <is>
+          <t>Tests</t>
+        </is>
+      </c>
+      <c r="D1401" t="inlineStr">
+        <is>
+          <t>Configurateurs &amp; coût de possession</t>
+        </is>
+      </c>
+      <c r="E1401" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="I1401" t="inlineStr">
+        <is>
+          <t>/tests/configurateurs-cout-de-possession/dacia-sandero-vs-clio-vi-prix-reel/</t>
+        </is>
+      </c>
+      <c r="J1401" t="inlineStr">
+        <is>
+          <t>B — Marques, essais &amp; sport auto</t>
+        </is>
+      </c>
+      <c r="K1401" t="inlineStr">
+        <is>
+          <t>en rédaction</t>
+        </is>
+      </c>
+    </row>
+    <row r="1402">
+      <c r="A1402" t="inlineStr">
+        <is>
+          <t>dacia duster vs peugeot 2008</t>
+        </is>
+      </c>
+      <c r="B1402" t="inlineStr">
+        <is>
+          <t>prix réel dacia duster 2026;prix réel peugeot 2008 2026;suv compact le moins cher 2026;coût de possession suv compact 2026</t>
+        </is>
+      </c>
+      <c r="C1402" t="inlineStr">
+        <is>
+          <t>Combien ça coûte vraiment</t>
+        </is>
+      </c>
+      <c r="D1402" t="inlineStr">
+        <is>
+          <t>Configurateurs &amp; coût de possession</t>
+        </is>
+      </c>
+      <c r="E1402" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="I1402" t="inlineStr">
+        <is>
+          <t>/combien-ca-coute-vraiment/configurateurs-cout-de-possession/duster-2008-cout-possession/</t>
+        </is>
+      </c>
+      <c r="J1402" t="inlineStr">
+        <is>
+          <t>B — Marques, essais &amp; sport auto</t>
+        </is>
+      </c>
+      <c r="K1402" t="inlineStr">
+        <is>
+          <t>en rédaction</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>